<commit_message>
SA Batch 1 Apollo enrichment (35 contacts, 16 companies) into Excel
</commit_message>
<xml_diff>
--- a/market-research/south-africa/I-MAK_SouthAfrica_Batch1_Food.xlsx
+++ b/market-research/south-africa/I-MAK_SouthAfrica_Batch1_Food.xlsx
@@ -12,7 +12,8 @@
     <sheet name="Top Prospects" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="By Industry" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="By Region" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Gearbox Suppliers" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Decision Makers" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Gearbox Suppliers" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,6 +56,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="002E5496"/>
     </font>
     <font>
       <i val="1"/>
@@ -125,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -152,7 +158,14 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6938,6 +6951,1539 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Full Name</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Business Email</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Email Status</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn URL</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Filmatic Packaging</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Riaan Van Zyl</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>rvanzyl@filmatic.com</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/riaan-van-zyl-41355240</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Cape Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Filmatic Packaging</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Chris Mijburgh</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Operations Director</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>chrism@filmatic.com</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/chris-mijburgh-850b193b</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Acepak</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Matthew Grobler</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>matthew@acepak.co.za</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/matthew-grobler-acepak</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Cape Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Acepak</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Clinton Meadows</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Technical Director</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>clinton@acepak.co.za</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/clinton-meadows-67807470</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Cape Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Acepak</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Justin Tomsett</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Sales Director</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>justin@acepak.co.za</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/justin-tomsett-acepak</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Cape Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Macadams International</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>John Reilly</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Chief Executive Officer</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>jreilly@macadams.co.za</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/john-reilly-5b841b23</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Johannesburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Macadams International</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Bruce Armstrong</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>barmstrong@macadams.co.za</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/bruce-armstrong-2793a4b2</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Durban</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Macadams International</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Projects/Technical</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Michael Hodgson</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Projects Director</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>mhodgson@macadams.co.za</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/michael-hodgson-a0a8182b</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Macadams International</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Neo Nkadimeng</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Production Manager</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>nnkadimeng@macadams.co.za</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/neo-nkadimeng-90ba7ba7</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Cape Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Macadams International</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Purchasing</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Selina Plaatjes</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Import Buying Manager</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>splaatjes@macadams.co.za</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/selina-plaatjes-805701282</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Cape Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>JF Equipment</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Francois Bester</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Operations Manager</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr"/>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/francois-bester-2b89561b5</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Anderson Engineering</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Hans Coertse</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>hans@andersoneng.co.za</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/hans-coertse-b4046070</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Durban</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Anderson Engineering</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Hennie Jager</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>henniedj@andersoneng.co.za</t>
+        </is>
+      </c>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/hpdejager</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Durban</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Anderson Engineering</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Andrew Charters</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Design Engineering Manager</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr"/>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/andrew-charters-097352bb</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Anderson Engineering</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Trevor Govender</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Operations Manager</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr"/>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/trevor-govender-2519a315</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Pietermaritzburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Facet Engineering</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Nicole Fairweather</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Operations Director</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>nicolefairweather@facetengineering.co.za</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/nicole-fairweather-910a4315</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Johannesburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Facet Engineering</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Johan Pretorius</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Technical Director</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr"/>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/johan-pretorius-798a3245</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Johannesburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Jones Industrial Mixers</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Gareth Lyndon</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Engineering Director</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>gareth@jonesmixers.co.za</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/gareth-lyndon-45b217a6</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Johannesburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Jones Industrial Mixers</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>John Broli</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr"/>
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/john-broli-46580217</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Johannesburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>CFAM Technologies</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Purchasing</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Riaan Redelinghuys</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Procurement Manager</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>riaan@cfam.co.za</t>
+        </is>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/riaan-redelinghuys-1959a228</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>National Packaging Systems (NPS)</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>John Pelucci</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>john@nps.co.za</t>
+        </is>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/john-pelucci-65b9084</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Durban</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>National Packaging Systems (NPS)</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Sanjay Sookdeo</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Operation Director</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>sanjay@nationalpackagingsystems.co.za</t>
+        </is>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/sanjay-sookdeo-29791899</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Durban</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Schullpak CC</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Graham Hull</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>graham@schullpak.co.za</t>
+        </is>
+      </c>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/graham-hull-54549b54</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>Cape Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Schullpak CC</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Operations/GM</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Johan Slabbert</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Operations / General Manager</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>johan@schullpak.co.za</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/johan-slabbert-20391a127</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Johannesburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Mixtec</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Jono Lyndon</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>jlyndon@mixtec.com</t>
+        </is>
+      </c>
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/jono-lyndon-78b6222a</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>Mixtec</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Metta Hofmeister</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr"/>
+      <c r="F27" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/metta-jan-hofmeister-4411653b</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Johannesburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Afromix (AFX Holdings)</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Eugene Els</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>eugene.els@afromix.co.za</t>
+        </is>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/eugene-els-166b1314</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>Johannesburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Afromix (AFX Holdings)</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Projects</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>JJ Strydom</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Projects Director</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>jj.strydom@afromix.co.za</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/jj-strydom-0a5b0347</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Johannesburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Afromix (AFX Holdings)</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Barry Middleton</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Financial Director</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>barry.middleton@afromix.co.za</t>
+        </is>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/barry-middleton-b63481220</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>Benoni</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>Afromix (AFX Holdings)</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Verna Els</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Sales and Marketing Director</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>verna.els@afromix.co.za</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/verna-els-203a97154</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Johannesburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>PMD Packaging</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Pat Galleymore</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Technical Director</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>pat@pmdpackaging.co.za</t>
+        </is>
+      </c>
+      <c r="F32" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/pat-galleymore-4971ba12a</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Inpakt Group</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Marketing/MD</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Nishara Naidoo</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Marketing Director (also MD Inpaktsa)</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>nishara@inpaktgroup.co.za</t>
+        </is>
+      </c>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/nishara-naidoo-95a39226</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Durban</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Basils Business Opportunities (BBO)</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Basil Phupha</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>basil@bbosa.co.za</t>
+        </is>
+      </c>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/basil-phupha-a41857197</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>Johannesburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Saturn Stainless Industries</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Jacques Schreuder</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>jacques@saturnstainless.co.za</t>
+        </is>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/jacques-schreuder-0aba4925</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Cape Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Saturn Stainless Industries</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Francois Carolissen</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Production Manager</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>francois@saturnstainless.co.za</t>
+        </is>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/francois-carolissen-15115a246</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>Paarl</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>35 decision-makers enriched via Apollo (16 of 42 companies). 29 verified business emails; rest email-unavailable (LinkedIn still provided).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="15" t="inlineStr">
+        <is>
+          <t>SA Apollo coverage is thin: 26 of 42 companies had NO records (incl. Roff, Powercon, Egli, MPE, STEGEL, Maize Master, Drotsky). For those use company website / LinkedIn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="15" t="inlineStr">
+        <is>
+          <t>EXCLUDED: ABC Hansen Africa's 2 Apollo matches were mis-linked to 'Argon Asset Management' (wrong org) and dropped.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -7102,7 +8648,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>All attributions INFERRED (no public BOM) except Mechaneer (documents worm-gear) &amp; Mixtec (openly multi-sources). SEW is the primary account incumbent.</t>
         </is>

</xml_diff>